<commit_message>
Update export samples (PDF + XLSX) with alignment and totals fixes
</commit_message>
<xml_diff>
--- a/export-despesas-sample.xlsx
+++ b/export-despesas-sample.xlsx
@@ -162,12 +162,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -519,195 +525,195 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="6">
         <v>130.8</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="6">
         <v>30.08</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="6">
         <v>160.88</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="6">
         <v>75.03</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="6">
         <v>18.49</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="6">
         <v>93.52</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="6">
         <v>52.03</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="6">
         <v>11.97</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="6">
         <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="6">
         <v>18.06</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="6">
         <v>1.08</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="6">
         <v>19.14</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="6">
         <v>52.03</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="6">
         <v>11.97</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="6">
         <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="6">
         <v>17.44</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="6">
         <v>4.01</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="6">
         <v>21.45</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="6">
         <v>17.44</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="6">
         <v>4.01</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="6">
         <v>21.45</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="6">
         <v>16.35</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="6">
         <v>3.76</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="6">
         <v>20.11</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="6">
         <v>16.35</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="6">
         <v>3.76</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="6">
         <v>20.11</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="6">
         <v>32.01</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="6">
         <v>7.36</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="6">
         <v>39.37</v>
       </c>
     </row>
@@ -727,38 +733,38 @@
     <col min="2" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="7" t="s">
         <v>30</v>
       </c>
     </row>
@@ -766,34 +772,34 @@
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -801,34 +807,34 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="5" t="s">
         <v>19</v>
       </c>
     </row>
@@ -836,34 +842,34 @@
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="6">
         <v>130.8</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="6">
         <v>75.03</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="6">
         <v>52.03</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="6">
         <v>18.06</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="6">
         <v>52.03</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="6">
         <v>17.44</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="6">
         <v>17.44</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="6">
         <v>16.35</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="6">
         <v>16.35</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="6">
         <v>32.01</v>
       </c>
     </row>
@@ -871,34 +877,34 @@
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="6">
         <v>30.08</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="6">
         <v>18.49</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="6">
         <v>11.97</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="6">
         <v>1.08</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="6">
         <v>11.97</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="6">
         <v>4.01</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="6">
         <v>4.01</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="6">
         <v>3.76</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="6">
         <v>3.76</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="6">
         <v>7.36</v>
       </c>
     </row>
@@ -906,34 +912,34 @@
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="6">
         <v>160.88</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="6">
         <v>93.52</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="6">
         <v>64</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="6">
         <v>19.14</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="6">
         <v>64</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="6">
         <v>21.45</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="6">
         <v>21.45</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="6">
         <v>20.11</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="6">
         <v>20.11</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="6">
         <v>39.37</v>
       </c>
     </row>

</xml_diff>